<commit_message>
Fix input filename: auto-detect both naming variants
Supports both '1000 + 86 клиник.xlsx' and '1000+86.xlsx'.

https://claude.ai/code/session_01RirjgdbnRw5p1vyEh4svFF
</commit_message>
<xml_diff>
--- a/1000+86.xlsx
+++ b/1000+86.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adelmustafina/Desktop/firecrawl-test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6902DA0-61D5-4644-BA0F-2524718B7A85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{283F29D4-F11F-2846-984D-AD9D5117E7DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="21260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4155" uniqueCount="3874">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4020" uniqueCount="3874">
   <si>
     <t>12К — психологический центр для родителей и детей</t>
   </si>
@@ -11853,7 +11853,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -11895,29 +11895,19 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="6">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <name val="Roboto"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -11934,6 +11924,24 @@
         <name val="Arial"/>
         <family val="2"/>
         <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <name val="Roboto"/>
+        <scheme val="none"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -12006,9 +12014,9 @@
   <tableColumns count="5">
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Name"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="URL"/>
-    <tableColumn id="9" xr3:uid="{E8C4287C-5A78-534A-950E-5866C2172739}" name="Description" dataDxfId="0"/>
+    <tableColumn id="9" xr3:uid="{E8C4287C-5A78-534A-950E-5866C2172739}" name="Description" dataDxfId="1"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Emails"/>
-    <tableColumn id="7" xr3:uid="{57A507DB-C489-C24B-8597-39C5E21513C7}" name="Phones" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{57A507DB-C489-C24B-8597-39C5E21513C7}" name="Phones" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="psychology_centers_moscow-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -12215,7 +12223,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:K1000"/>
+  <dimension ref="A1:M1000"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="36.5" customWidth="1"/>
@@ -12223,7 +12231,7 @@
     <col min="4" max="5" width="22.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>235</v>
       </c>
@@ -12258,7 +12266,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -12270,8 +12278,16 @@
         <v>2</v>
       </c>
       <c r="E2" s="2"/>
-    </row>
-    <row r="3" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="19"/>
+      <c r="L2" s="19"/>
+      <c r="M2" s="19"/>
+    </row>
+    <row r="3" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
@@ -12283,26 +12299,16 @@
         <v>5</v>
       </c>
       <c r="E3" s="2"/>
-      <c r="F3" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="G3" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="H3" s="10">
-        <v>100</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>254</v>
-      </c>
-      <c r="J3" s="11" t="s">
-        <v>255</v>
-      </c>
-      <c r="K3" s="7" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="20"/>
+      <c r="K3" s="20"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+    </row>
+    <row r="4" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -12314,14 +12320,16 @@
         <v>8</v>
       </c>
       <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-    </row>
-    <row r="5" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
+      <c r="I4" s="22"/>
+      <c r="J4" s="22"/>
+      <c r="K4" s="22"/>
+      <c r="L4" s="19"/>
+      <c r="M4" s="19"/>
+    </row>
+    <row r="5" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
@@ -12333,14 +12341,16 @@
         <v>11</v>
       </c>
       <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-    </row>
-    <row r="6" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="22"/>
+      <c r="J5" s="22"/>
+      <c r="K5" s="22"/>
+      <c r="L5" s="19"/>
+      <c r="M5" s="19"/>
+    </row>
+    <row r="6" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
@@ -12352,14 +12362,16 @@
         <v>14</v>
       </c>
       <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
-    </row>
-    <row r="7" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F6" s="22"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="22"/>
+      <c r="I6" s="22"/>
+      <c r="J6" s="22"/>
+      <c r="K6" s="22"/>
+      <c r="L6" s="19"/>
+      <c r="M6" s="19"/>
+    </row>
+    <row r="7" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="2" t="s">
         <v>15</v>
       </c>
@@ -12371,14 +12383,16 @@
         <v>17</v>
       </c>
       <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
-    </row>
-    <row r="8" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F7" s="22"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="22"/>
+      <c r="I7" s="22"/>
+      <c r="J7" s="22"/>
+      <c r="K7" s="22"/>
+      <c r="L7" s="19"/>
+      <c r="M7" s="19"/>
+    </row>
+    <row r="8" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="2" t="s">
         <v>18</v>
       </c>
@@ -12390,14 +12404,16 @@
         <v>20</v>
       </c>
       <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-    </row>
-    <row r="9" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F8" s="22"/>
+      <c r="G8" s="22"/>
+      <c r="H8" s="22"/>
+      <c r="I8" s="22"/>
+      <c r="J8" s="22"/>
+      <c r="K8" s="22"/>
+      <c r="L8" s="19"/>
+      <c r="M8" s="19"/>
+    </row>
+    <row r="9" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="2" t="s">
         <v>21</v>
       </c>
@@ -12409,26 +12425,16 @@
         <v>23</v>
       </c>
       <c r="E9" s="2"/>
-      <c r="F9" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="G9" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="H9" s="10">
-        <v>100</v>
-      </c>
-      <c r="I9" s="7" t="s">
-        <v>284</v>
-      </c>
-      <c r="J9" s="9" t="s">
-        <v>285</v>
-      </c>
-      <c r="K9" s="7" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="21"/>
+      <c r="I9" s="20"/>
+      <c r="J9" s="20"/>
+      <c r="K9" s="20"/>
+      <c r="L9" s="19"/>
+      <c r="M9" s="19"/>
+    </row>
+    <row r="10" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="2" t="s">
         <v>24</v>
       </c>
@@ -12440,14 +12446,16 @@
         <v>26</v>
       </c>
       <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-    </row>
-    <row r="11" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F10" s="22"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="22"/>
+      <c r="I10" s="22"/>
+      <c r="J10" s="22"/>
+      <c r="K10" s="22"/>
+      <c r="L10" s="19"/>
+      <c r="M10" s="19"/>
+    </row>
+    <row r="11" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="2" t="s">
         <v>27</v>
       </c>
@@ -12459,26 +12467,16 @@
         <v>29</v>
       </c>
       <c r="E11" s="2"/>
-      <c r="F11" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="G11" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="H11" s="10">
-        <v>100</v>
-      </c>
-      <c r="I11" s="7" t="s">
-        <v>295</v>
-      </c>
-      <c r="J11" s="9" t="s">
-        <v>285</v>
-      </c>
-      <c r="K11" s="7" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F11" s="20"/>
+      <c r="G11" s="20"/>
+      <c r="H11" s="21"/>
+      <c r="I11" s="20"/>
+      <c r="J11" s="20"/>
+      <c r="K11" s="20"/>
+      <c r="L11" s="19"/>
+      <c r="M11" s="19"/>
+    </row>
+    <row r="12" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="2" t="s">
         <v>30</v>
       </c>
@@ -12490,26 +12488,16 @@
         <v>32</v>
       </c>
       <c r="E12" s="2"/>
-      <c r="F12" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="G12" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="H12" s="10">
-        <v>100</v>
-      </c>
-      <c r="I12" s="7" t="s">
-        <v>301</v>
-      </c>
-      <c r="J12" s="9" t="s">
-        <v>285</v>
-      </c>
-      <c r="K12" s="7" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F12" s="20"/>
+      <c r="G12" s="20"/>
+      <c r="H12" s="21"/>
+      <c r="I12" s="20"/>
+      <c r="J12" s="20"/>
+      <c r="K12" s="20"/>
+      <c r="L12" s="19"/>
+      <c r="M12" s="19"/>
+    </row>
+    <row r="13" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="2" t="s">
         <v>33</v>
       </c>
@@ -12521,26 +12509,16 @@
         <v>35</v>
       </c>
       <c r="E13" s="2"/>
-      <c r="F13" s="13" t="s">
-        <v>307</v>
-      </c>
-      <c r="G13" s="13" t="s">
-        <v>308</v>
-      </c>
-      <c r="H13" s="10">
-        <v>0</v>
-      </c>
-      <c r="I13" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="J13" s="13" t="s">
-        <v>310</v>
-      </c>
-      <c r="K13" s="7" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F13" s="20"/>
+      <c r="G13" s="20"/>
+      <c r="H13" s="21"/>
+      <c r="I13" s="20"/>
+      <c r="J13" s="20"/>
+      <c r="K13" s="20"/>
+      <c r="L13" s="19"/>
+      <c r="M13" s="19"/>
+    </row>
+    <row r="14" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="2" t="s">
         <v>36</v>
       </c>
@@ -12552,26 +12530,16 @@
         <v>38</v>
       </c>
       <c r="E14" s="2"/>
-      <c r="F14" s="13" t="s">
-        <v>307</v>
-      </c>
-      <c r="G14" s="13" t="s">
-        <v>308</v>
-      </c>
-      <c r="H14" s="10">
-        <v>0</v>
-      </c>
-      <c r="I14" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="J14" s="13" t="s">
-        <v>310</v>
-      </c>
-      <c r="K14" s="7" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F14" s="20"/>
+      <c r="G14" s="20"/>
+      <c r="H14" s="21"/>
+      <c r="I14" s="20"/>
+      <c r="J14" s="20"/>
+      <c r="K14" s="20"/>
+      <c r="L14" s="19"/>
+      <c r="M14" s="19"/>
+    </row>
+    <row r="15" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="2" t="s">
         <v>39</v>
       </c>
@@ -12583,14 +12551,16 @@
         <v>41</v>
       </c>
       <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
-    </row>
-    <row r="16" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F15" s="22"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="22"/>
+      <c r="I15" s="22"/>
+      <c r="J15" s="22"/>
+      <c r="K15" s="22"/>
+      <c r="L15" s="19"/>
+      <c r="M15" s="19"/>
+    </row>
+    <row r="16" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="2" t="s">
         <v>42</v>
       </c>
@@ -12602,14 +12572,16 @@
         <v>44</v>
       </c>
       <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
-    </row>
-    <row r="17" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F16" s="22"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="22"/>
+      <c r="I16" s="22"/>
+      <c r="J16" s="22"/>
+      <c r="K16" s="22"/>
+      <c r="L16" s="19"/>
+      <c r="M16" s="19"/>
+    </row>
+    <row r="17" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="2" t="s">
         <v>45</v>
       </c>
@@ -12621,26 +12593,16 @@
         <v>47</v>
       </c>
       <c r="E17" s="2"/>
-      <c r="F17" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="G17" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="H17" s="10">
-        <v>100</v>
-      </c>
-      <c r="I17" s="7" t="s">
-        <v>326</v>
-      </c>
-      <c r="J17" s="13" t="s">
-        <v>310</v>
-      </c>
-      <c r="K17" s="7" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F17" s="20"/>
+      <c r="G17" s="20"/>
+      <c r="H17" s="21"/>
+      <c r="I17" s="20"/>
+      <c r="J17" s="20"/>
+      <c r="K17" s="20"/>
+      <c r="L17" s="19"/>
+      <c r="M17" s="19"/>
+    </row>
+    <row r="18" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="2" t="s">
         <v>48</v>
       </c>
@@ -12652,26 +12614,16 @@
         <v>50</v>
       </c>
       <c r="E18" s="2"/>
-      <c r="F18" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="G18" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="H18" s="10">
-        <v>100</v>
-      </c>
-      <c r="I18" s="7" t="s">
-        <v>331</v>
-      </c>
-      <c r="J18" s="9" t="s">
-        <v>285</v>
-      </c>
-      <c r="K18" s="7" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F18" s="20"/>
+      <c r="G18" s="20"/>
+      <c r="H18" s="21"/>
+      <c r="I18" s="20"/>
+      <c r="J18" s="20"/>
+      <c r="K18" s="20"/>
+      <c r="L18" s="19"/>
+      <c r="M18" s="19"/>
+    </row>
+    <row r="19" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="2" t="s">
         <v>51</v>
       </c>
@@ -12683,26 +12635,16 @@
         <v>53</v>
       </c>
       <c r="E19" s="2"/>
-      <c r="F19" s="11" t="s">
-        <v>336</v>
-      </c>
-      <c r="G19" s="13" t="s">
-        <v>308</v>
-      </c>
-      <c r="H19" s="10">
-        <v>0</v>
-      </c>
-      <c r="I19" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="J19" s="13" t="s">
-        <v>310</v>
-      </c>
-      <c r="K19" s="7" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F19" s="20"/>
+      <c r="G19" s="20"/>
+      <c r="H19" s="21"/>
+      <c r="I19" s="20"/>
+      <c r="J19" s="20"/>
+      <c r="K19" s="20"/>
+      <c r="L19" s="19"/>
+      <c r="M19" s="19"/>
+    </row>
+    <row r="20" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="2" t="s">
         <v>54</v>
       </c>
@@ -12714,26 +12656,16 @@
         <v>56</v>
       </c>
       <c r="E20" s="2"/>
-      <c r="F20" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="G20" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="H20" s="10">
-        <v>100</v>
-      </c>
-      <c r="I20" s="7" t="s">
-        <v>340</v>
-      </c>
-      <c r="J20" s="13" t="s">
-        <v>310</v>
-      </c>
-      <c r="K20" s="7" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F20" s="20"/>
+      <c r="G20" s="20"/>
+      <c r="H20" s="21"/>
+      <c r="I20" s="20"/>
+      <c r="J20" s="20"/>
+      <c r="K20" s="20"/>
+      <c r="L20" s="19"/>
+      <c r="M20" s="19"/>
+    </row>
+    <row r="21" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="2" t="s">
         <v>57</v>
       </c>
@@ -12745,14 +12677,16 @@
         <v>59</v>
       </c>
       <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
-      <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
-      <c r="J21" s="2"/>
-      <c r="K21" s="2"/>
-    </row>
-    <row r="22" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F21" s="22"/>
+      <c r="G21" s="22"/>
+      <c r="H21" s="22"/>
+      <c r="I21" s="22"/>
+      <c r="J21" s="22"/>
+      <c r="K21" s="22"/>
+      <c r="L21" s="19"/>
+      <c r="M21" s="19"/>
+    </row>
+    <row r="22" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="2" t="s">
         <v>60</v>
       </c>
@@ -12764,26 +12698,16 @@
         <v>62</v>
       </c>
       <c r="E22" s="2"/>
-      <c r="F22" s="11" t="s">
-        <v>336</v>
-      </c>
-      <c r="G22" s="13" t="s">
-        <v>308</v>
-      </c>
-      <c r="H22" s="10">
-        <v>0</v>
-      </c>
-      <c r="I22" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="J22" s="13" t="s">
-        <v>310</v>
-      </c>
-      <c r="K22" s="7" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F22" s="20"/>
+      <c r="G22" s="20"/>
+      <c r="H22" s="21"/>
+      <c r="I22" s="20"/>
+      <c r="J22" s="20"/>
+      <c r="K22" s="20"/>
+      <c r="L22" s="19"/>
+      <c r="M22" s="19"/>
+    </row>
+    <row r="23" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="2" t="s">
         <v>63</v>
       </c>
@@ -12795,26 +12719,16 @@
         <v>65</v>
       </c>
       <c r="E23" s="2"/>
-      <c r="F23" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="G23" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="H23" s="10">
-        <v>100</v>
-      </c>
-      <c r="I23" s="7" t="s">
-        <v>354</v>
-      </c>
-      <c r="J23" s="9" t="s">
-        <v>285</v>
-      </c>
-      <c r="K23" s="7" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F23" s="20"/>
+      <c r="G23" s="20"/>
+      <c r="H23" s="21"/>
+      <c r="I23" s="20"/>
+      <c r="J23" s="20"/>
+      <c r="K23" s="20"/>
+      <c r="L23" s="19"/>
+      <c r="M23" s="19"/>
+    </row>
+    <row r="24" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="2" t="s">
         <v>66</v>
       </c>
@@ -12826,26 +12740,16 @@
         <v>68</v>
       </c>
       <c r="E24" s="2"/>
-      <c r="F24" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="G24" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="H24" s="10">
-        <v>100</v>
-      </c>
-      <c r="I24" s="7" t="s">
-        <v>340</v>
-      </c>
-      <c r="J24" s="9" t="s">
-        <v>285</v>
-      </c>
-      <c r="K24" s="7" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F24" s="20"/>
+      <c r="G24" s="20"/>
+      <c r="H24" s="21"/>
+      <c r="I24" s="20"/>
+      <c r="J24" s="20"/>
+      <c r="K24" s="20"/>
+      <c r="L24" s="19"/>
+      <c r="M24" s="19"/>
+    </row>
+    <row r="25" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="2" t="s">
         <v>69</v>
       </c>
@@ -12857,26 +12761,16 @@
         <v>71</v>
       </c>
       <c r="E25" s="2"/>
-      <c r="F25" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="G25" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="H25" s="10">
-        <v>100</v>
-      </c>
-      <c r="I25" s="7" t="s">
-        <v>365</v>
-      </c>
-      <c r="J25" s="9" t="s">
-        <v>285</v>
-      </c>
-      <c r="K25" s="7" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F25" s="20"/>
+      <c r="G25" s="20"/>
+      <c r="H25" s="21"/>
+      <c r="I25" s="20"/>
+      <c r="J25" s="20"/>
+      <c r="K25" s="20"/>
+      <c r="L25" s="19"/>
+      <c r="M25" s="19"/>
+    </row>
+    <row r="26" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="2" t="s">
         <v>72</v>
       </c>
@@ -12888,26 +12782,16 @@
         <v>74</v>
       </c>
       <c r="E26" s="2"/>
-      <c r="F26" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="G26" s="11" t="s">
-        <v>369</v>
-      </c>
-      <c r="H26" s="10">
-        <v>0</v>
-      </c>
-      <c r="I26" s="7" t="s">
-        <v>370</v>
-      </c>
-      <c r="J26" s="13" t="s">
-        <v>310</v>
-      </c>
-      <c r="K26" s="7" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F26" s="20"/>
+      <c r="G26" s="20"/>
+      <c r="H26" s="21"/>
+      <c r="I26" s="20"/>
+      <c r="J26" s="20"/>
+      <c r="K26" s="20"/>
+      <c r="L26" s="19"/>
+      <c r="M26" s="19"/>
+    </row>
+    <row r="27" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="2" t="s">
         <v>75</v>
       </c>
@@ -12919,14 +12803,16 @@
         <v>77</v>
       </c>
       <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="2"/>
-      <c r="I27" s="2"/>
-      <c r="J27" s="2"/>
-      <c r="K27" s="2"/>
-    </row>
-    <row r="28" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F27" s="22"/>
+      <c r="G27" s="22"/>
+      <c r="H27" s="22"/>
+      <c r="I27" s="22"/>
+      <c r="J27" s="22"/>
+      <c r="K27" s="22"/>
+      <c r="L27" s="19"/>
+      <c r="M27" s="19"/>
+    </row>
+    <row r="28" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="2" t="s">
         <v>78</v>
       </c>
@@ -12938,26 +12824,16 @@
         <v>80</v>
       </c>
       <c r="E28" s="2"/>
-      <c r="F28" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="G28" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="H28" s="10">
-        <v>100</v>
-      </c>
-      <c r="I28" s="7" t="s">
-        <v>380</v>
-      </c>
-      <c r="J28" s="13" t="s">
-        <v>310</v>
-      </c>
-      <c r="K28" s="7" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F28" s="20"/>
+      <c r="G28" s="20"/>
+      <c r="H28" s="21"/>
+      <c r="I28" s="20"/>
+      <c r="J28" s="20"/>
+      <c r="K28" s="20"/>
+      <c r="L28" s="19"/>
+      <c r="M28" s="19"/>
+    </row>
+    <row r="29" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="2" t="s">
         <v>81</v>
       </c>
@@ -12969,26 +12845,16 @@
         <v>83</v>
       </c>
       <c r="E29" s="2"/>
-      <c r="F29" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="G29" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="H29" s="10">
-        <v>100</v>
-      </c>
-      <c r="I29" s="7" t="s">
-        <v>385</v>
-      </c>
-      <c r="J29" s="9" t="s">
-        <v>285</v>
-      </c>
-      <c r="K29" s="7" t="s">
-        <v>386</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F29" s="20"/>
+      <c r="G29" s="20"/>
+      <c r="H29" s="21"/>
+      <c r="I29" s="20"/>
+      <c r="J29" s="20"/>
+      <c r="K29" s="20"/>
+      <c r="L29" s="19"/>
+      <c r="M29" s="19"/>
+    </row>
+    <row r="30" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="2" t="s">
         <v>84</v>
       </c>
@@ -13000,26 +12866,16 @@
         <v>86</v>
       </c>
       <c r="E30" s="2"/>
-      <c r="F30" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="G30" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="H30" s="10">
-        <v>100</v>
-      </c>
-      <c r="I30" s="7" t="s">
-        <v>340</v>
-      </c>
-      <c r="J30" s="9" t="s">
-        <v>285</v>
-      </c>
-      <c r="K30" s="7" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F30" s="20"/>
+      <c r="G30" s="20"/>
+      <c r="H30" s="21"/>
+      <c r="I30" s="20"/>
+      <c r="J30" s="20"/>
+      <c r="K30" s="20"/>
+      <c r="L30" s="19"/>
+      <c r="M30" s="19"/>
+    </row>
+    <row r="31" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="2" t="s">
         <v>87</v>
       </c>
@@ -13031,26 +12887,16 @@
         <v>89</v>
       </c>
       <c r="E31" s="2"/>
-      <c r="F31" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="G31" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="H31" s="10">
-        <v>100</v>
-      </c>
-      <c r="I31" s="7" t="s">
-        <v>331</v>
-      </c>
-      <c r="J31" s="11" t="s">
-        <v>255</v>
-      </c>
-      <c r="K31" s="7" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F31" s="20"/>
+      <c r="G31" s="20"/>
+      <c r="H31" s="21"/>
+      <c r="I31" s="20"/>
+      <c r="J31" s="20"/>
+      <c r="K31" s="20"/>
+      <c r="L31" s="19"/>
+      <c r="M31" s="19"/>
+    </row>
+    <row r="32" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="2" t="s">
         <v>90</v>
       </c>
@@ -13062,14 +12908,16 @@
         <v>92</v>
       </c>
       <c r="E32" s="2"/>
-      <c r="F32" s="2"/>
-      <c r="G32" s="2"/>
-      <c r="H32" s="2"/>
-      <c r="I32" s="2"/>
-      <c r="J32" s="2"/>
-      <c r="K32" s="2"/>
-    </row>
-    <row r="33" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F32" s="22"/>
+      <c r="G32" s="22"/>
+      <c r="H32" s="22"/>
+      <c r="I32" s="22"/>
+      <c r="J32" s="22"/>
+      <c r="K32" s="22"/>
+      <c r="L32" s="19"/>
+      <c r="M32" s="19"/>
+    </row>
+    <row r="33" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="2" t="s">
         <v>93</v>
       </c>
@@ -13081,14 +12929,16 @@
         <v>95</v>
       </c>
       <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
-      <c r="H33" s="2"/>
-      <c r="I33" s="2"/>
-      <c r="J33" s="2"/>
-      <c r="K33" s="2"/>
-    </row>
-    <row r="34" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F33" s="22"/>
+      <c r="G33" s="22"/>
+      <c r="H33" s="22"/>
+      <c r="I33" s="22"/>
+      <c r="J33" s="22"/>
+      <c r="K33" s="22"/>
+      <c r="L33" s="19"/>
+      <c r="M33" s="19"/>
+    </row>
+    <row r="34" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A34" s="2" t="s">
         <v>96</v>
       </c>
@@ -13100,14 +12950,16 @@
         <v>98</v>
       </c>
       <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-      <c r="G34" s="2"/>
-      <c r="H34" s="2"/>
-      <c r="I34" s="2"/>
-      <c r="J34" s="2"/>
-      <c r="K34" s="2"/>
-    </row>
-    <row r="35" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F34" s="22"/>
+      <c r="G34" s="22"/>
+      <c r="H34" s="22"/>
+      <c r="I34" s="22"/>
+      <c r="J34" s="22"/>
+      <c r="K34" s="22"/>
+      <c r="L34" s="19"/>
+      <c r="M34" s="19"/>
+    </row>
+    <row r="35" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A35" s="2" t="s">
         <v>99</v>
       </c>
@@ -13119,26 +12971,16 @@
         <v>101</v>
       </c>
       <c r="E35" s="2"/>
-      <c r="F35" s="11" t="s">
-        <v>336</v>
-      </c>
-      <c r="G35" s="13" t="s">
-        <v>308</v>
-      </c>
-      <c r="H35" s="10">
-        <v>0</v>
-      </c>
-      <c r="I35" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="J35" s="13" t="s">
-        <v>310</v>
-      </c>
-      <c r="K35" s="7" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F35" s="20"/>
+      <c r="G35" s="20"/>
+      <c r="H35" s="21"/>
+      <c r="I35" s="20"/>
+      <c r="J35" s="20"/>
+      <c r="K35" s="20"/>
+      <c r="L35" s="19"/>
+      <c r="M35" s="19"/>
+    </row>
+    <row r="36" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A36" s="2" t="s">
         <v>102</v>
       </c>
@@ -13150,26 +12992,16 @@
         <v>104</v>
       </c>
       <c r="E36" s="2"/>
-      <c r="F36" s="11" t="s">
-        <v>336</v>
-      </c>
-      <c r="G36" s="13" t="s">
-        <v>308</v>
-      </c>
-      <c r="H36" s="10">
-        <v>0</v>
-      </c>
-      <c r="I36" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="J36" s="13" t="s">
-        <v>310</v>
-      </c>
-      <c r="K36" s="7" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F36" s="20"/>
+      <c r="G36" s="20"/>
+      <c r="H36" s="21"/>
+      <c r="I36" s="20"/>
+      <c r="J36" s="20"/>
+      <c r="K36" s="20"/>
+      <c r="L36" s="19"/>
+      <c r="M36" s="19"/>
+    </row>
+    <row r="37" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A37" s="2" t="s">
         <v>105</v>
       </c>
@@ -13181,14 +13013,16 @@
         <v>107</v>
       </c>
       <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
-      <c r="G37" s="2"/>
-      <c r="H37" s="2"/>
-      <c r="I37" s="2"/>
-      <c r="J37" s="2"/>
-      <c r="K37" s="2"/>
-    </row>
-    <row r="38" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F37" s="22"/>
+      <c r="G37" s="22"/>
+      <c r="H37" s="22"/>
+      <c r="I37" s="22"/>
+      <c r="J37" s="22"/>
+      <c r="K37" s="22"/>
+      <c r="L37" s="19"/>
+      <c r="M37" s="19"/>
+    </row>
+    <row r="38" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A38" s="2" t="s">
         <v>108</v>
       </c>
@@ -13200,26 +13034,16 @@
         <v>110</v>
       </c>
       <c r="E38" s="2"/>
-      <c r="F38" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="G38" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="H38" s="10">
-        <v>100</v>
-      </c>
-      <c r="I38" s="7" t="s">
-        <v>426</v>
-      </c>
-      <c r="J38" s="11" t="s">
-        <v>255</v>
-      </c>
-      <c r="K38" s="7" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F38" s="20"/>
+      <c r="G38" s="20"/>
+      <c r="H38" s="21"/>
+      <c r="I38" s="20"/>
+      <c r="J38" s="20"/>
+      <c r="K38" s="20"/>
+      <c r="L38" s="19"/>
+      <c r="M38" s="19"/>
+    </row>
+    <row r="39" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A39" s="2" t="s">
         <v>111</v>
       </c>
@@ -13231,26 +13055,16 @@
         <v>113</v>
       </c>
       <c r="E39" s="2"/>
-      <c r="F39" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="G39" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="H39" s="10">
-        <v>100</v>
-      </c>
-      <c r="I39" s="7" t="s">
-        <v>432</v>
-      </c>
-      <c r="J39" s="13" t="s">
-        <v>310</v>
-      </c>
-      <c r="K39" s="7" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F39" s="20"/>
+      <c r="G39" s="20"/>
+      <c r="H39" s="21"/>
+      <c r="I39" s="20"/>
+      <c r="J39" s="20"/>
+      <c r="K39" s="20"/>
+      <c r="L39" s="19"/>
+      <c r="M39" s="19"/>
+    </row>
+    <row r="40" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A40" s="2" t="s">
         <v>114</v>
       </c>
@@ -13262,14 +13076,16 @@
         <v>116</v>
       </c>
       <c r="E40" s="2"/>
-      <c r="F40" s="2"/>
-      <c r="G40" s="2"/>
-      <c r="H40" s="2"/>
-      <c r="I40" s="2"/>
-      <c r="J40" s="2"/>
-      <c r="K40" s="2"/>
-    </row>
-    <row r="41" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F40" s="22"/>
+      <c r="G40" s="22"/>
+      <c r="H40" s="22"/>
+      <c r="I40" s="22"/>
+      <c r="J40" s="22"/>
+      <c r="K40" s="22"/>
+      <c r="L40" s="19"/>
+      <c r="M40" s="19"/>
+    </row>
+    <row r="41" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A41" s="2" t="s">
         <v>117</v>
       </c>
@@ -13281,26 +13097,16 @@
         <v>119</v>
       </c>
       <c r="E41" s="2"/>
-      <c r="F41" s="11" t="s">
-        <v>440</v>
-      </c>
-      <c r="G41" s="13" t="s">
-        <v>308</v>
-      </c>
-      <c r="H41" s="10">
-        <v>0</v>
-      </c>
-      <c r="I41" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="J41" s="13" t="s">
-        <v>310</v>
-      </c>
-      <c r="K41" s="7" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F41" s="20"/>
+      <c r="G41" s="20"/>
+      <c r="H41" s="21"/>
+      <c r="I41" s="20"/>
+      <c r="J41" s="20"/>
+      <c r="K41" s="20"/>
+      <c r="L41" s="19"/>
+      <c r="M41" s="19"/>
+    </row>
+    <row r="42" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A42" s="2" t="s">
         <v>120</v>
       </c>
@@ -13312,26 +13118,16 @@
         <v>122</v>
       </c>
       <c r="E42" s="2"/>
-      <c r="F42" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="G42" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="H42" s="10">
-        <v>100</v>
-      </c>
-      <c r="I42" s="7" t="s">
-        <v>284</v>
-      </c>
-      <c r="J42" s="11" t="s">
-        <v>255</v>
-      </c>
-      <c r="K42" s="7" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F42" s="20"/>
+      <c r="G42" s="20"/>
+      <c r="H42" s="21"/>
+      <c r="I42" s="20"/>
+      <c r="J42" s="20"/>
+      <c r="K42" s="20"/>
+      <c r="L42" s="19"/>
+      <c r="M42" s="19"/>
+    </row>
+    <row r="43" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A43" s="2" t="s">
         <v>123</v>
       </c>
@@ -13343,26 +13139,16 @@
         <v>125</v>
       </c>
       <c r="E43" s="2"/>
-      <c r="F43" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="G43" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="H43" s="10">
-        <v>100</v>
-      </c>
-      <c r="I43" s="7" t="s">
-        <v>284</v>
-      </c>
-      <c r="J43" s="9" t="s">
-        <v>285</v>
-      </c>
-      <c r="K43" s="7" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F43" s="20"/>
+      <c r="G43" s="20"/>
+      <c r="H43" s="21"/>
+      <c r="I43" s="20"/>
+      <c r="J43" s="20"/>
+      <c r="K43" s="20"/>
+      <c r="L43" s="19"/>
+      <c r="M43" s="19"/>
+    </row>
+    <row r="44" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A44" s="2" t="s">
         <v>126</v>
       </c>
@@ -13374,14 +13160,16 @@
         <v>128</v>
       </c>
       <c r="E44" s="2"/>
-      <c r="F44" s="2"/>
-      <c r="G44" s="2"/>
-      <c r="H44" s="2"/>
-      <c r="I44" s="2"/>
-      <c r="J44" s="2"/>
-      <c r="K44" s="2"/>
-    </row>
-    <row r="45" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F44" s="22"/>
+      <c r="G44" s="22"/>
+      <c r="H44" s="22"/>
+      <c r="I44" s="22"/>
+      <c r="J44" s="22"/>
+      <c r="K44" s="22"/>
+      <c r="L44" s="19"/>
+      <c r="M44" s="19"/>
+    </row>
+    <row r="45" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A45" s="2" t="s">
         <v>129</v>
       </c>
@@ -13393,26 +13181,16 @@
         <v>131</v>
       </c>
       <c r="E45" s="2"/>
-      <c r="F45" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="G45" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="H45" s="10">
-        <v>100</v>
-      </c>
-      <c r="I45" s="7" t="s">
-        <v>461</v>
-      </c>
-      <c r="J45" s="9" t="s">
-        <v>285</v>
-      </c>
-      <c r="K45" s="7" t="s">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F45" s="20"/>
+      <c r="G45" s="20"/>
+      <c r="H45" s="21"/>
+      <c r="I45" s="20"/>
+      <c r="J45" s="20"/>
+      <c r="K45" s="20"/>
+      <c r="L45" s="19"/>
+      <c r="M45" s="19"/>
+    </row>
+    <row r="46" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A46" s="2" t="s">
         <v>132</v>
       </c>
@@ -13424,14 +13202,16 @@
         <v>134</v>
       </c>
       <c r="E46" s="2"/>
-      <c r="F46" s="2"/>
-      <c r="G46" s="2"/>
-      <c r="H46" s="2"/>
-      <c r="I46" s="2"/>
-      <c r="J46" s="2"/>
-      <c r="K46" s="2"/>
-    </row>
-    <row r="47" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F46" s="22"/>
+      <c r="G46" s="22"/>
+      <c r="H46" s="22"/>
+      <c r="I46" s="22"/>
+      <c r="J46" s="22"/>
+      <c r="K46" s="22"/>
+      <c r="L46" s="19"/>
+      <c r="M46" s="19"/>
+    </row>
+    <row r="47" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A47" s="2" t="s">
         <v>135</v>
       </c>
@@ -13443,14 +13223,16 @@
         <v>137</v>
       </c>
       <c r="E47" s="2"/>
-      <c r="F47" s="2"/>
-      <c r="G47" s="2"/>
-      <c r="H47" s="2"/>
-      <c r="I47" s="2"/>
-      <c r="J47" s="2"/>
-      <c r="K47" s="2"/>
-    </row>
-    <row r="48" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F47" s="22"/>
+      <c r="G47" s="22"/>
+      <c r="H47" s="22"/>
+      <c r="I47" s="22"/>
+      <c r="J47" s="22"/>
+      <c r="K47" s="22"/>
+      <c r="L47" s="19"/>
+      <c r="M47" s="19"/>
+    </row>
+    <row r="48" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A48" s="2" t="s">
         <v>138</v>
       </c>

</xml_diff>